<commit_message>
Update Excel template columns to match form fields
- Simplified columns: Order No, Booking Date, Customer, Location, etc.
- Updated SAMPLE data structure with cleaner column names
- Updated column indices in upload and fetch logic
- Regenerated nrm-template.xlsx with new headers
- Makes bulk upload and single entry consistent
</commit_message>
<xml_diff>
--- a/public/nrm-template.xlsx
+++ b/public/nrm-template.xlsx
@@ -397,181 +397,103 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BD1"/>
+  <dimension ref="A1:V1"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="18.83203125" customWidth="1"/>
+    <col min="18" max="18" width="18.83203125" customWidth="1"/>
+    <col min="19" max="19" width="18.83203125" customWidth="1"/>
+    <col min="20" max="20" width="18.83203125" customWidth="1"/>
+    <col min="21" max="21" width="18.83203125" customWidth="1"/>
+    <col min="22" max="22" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>S.No</v>
+        <v>Order No</v>
       </c>
       <c r="B1" t="str">
-        <v>Purchase Inv No</v>
+        <v>Booking Date</v>
       </c>
       <c r="C1" t="str">
-        <v>Date of Purchase Invoice</v>
+        <v>Customer</v>
       </c>
       <c r="D1" t="str">
-        <v>Ageing</v>
+        <v>Location</v>
       </c>
       <c r="E1" t="str">
-        <v>Order_Number</v>
+        <v>Executive</v>
       </c>
       <c r="F1" t="str">
-        <v>Invoice_No</v>
+        <v>Team Leader</v>
       </c>
       <c r="G1" t="str">
-        <v>Invoice_Date</v>
+        <v>Make</v>
       </c>
       <c r="H1" t="str">
-        <v>Customer_Name</v>
+        <v>Variant</v>
       </c>
       <c r="I1" t="str">
-        <v>Chassis_No</v>
+        <v>Units</v>
       </c>
       <c r="J1" t="str">
-        <v>Team Leader</v>
+        <v>Chassis No</v>
       </c>
       <c r="K1" t="str">
-        <v>Location</v>
+        <v>Allotment Date</v>
       </c>
       <c r="L1" t="str">
-        <v>EXECUTIVE NAME</v>
+        <v>Invoice No</v>
       </c>
       <c r="M1" t="str">
-        <v xml:space="preserve"> Parent Product Line</v>
+        <v>Invoice Date</v>
       </c>
       <c r="N1" t="str">
-        <v>Make</v>
+        <v>Delivery Date</v>
       </c>
       <c r="O1" t="str">
-        <v>Nos.</v>
+        <v>Sales Price</v>
       </c>
       <c r="P1" t="str">
-        <v xml:space="preserve"> Product Line</v>
+        <v>Purchase Price</v>
       </c>
       <c r="Q1" t="str">
-        <v>Pre GST Sales Price</v>
+        <v>POD</v>
       </c>
       <c r="R1" t="str">
-        <v>Pre GST Purchases Price</v>
+        <v>Scheme Discount</v>
       </c>
       <c r="S1" t="str">
-        <v>POD</v>
+        <v>Additional Discount</v>
       </c>
       <c r="T1" t="str">
-        <v xml:space="preserve"> Gross Dealer Margin  </v>
+        <v>TML Discount</v>
       </c>
       <c r="U1" t="str">
-        <v xml:space="preserve"> Scheme discount </v>
+        <v>Other Income</v>
       </c>
       <c r="V1" t="str">
-        <v>Exchange</v>
-      </c>
-      <c r="W1" t="str">
-        <v>Corporate</v>
-      </c>
-      <c r="X1" t="str">
-        <v>Intervention</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>CSD</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>Scrappage</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>SSS</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>Price Diffrance</v>
-      </c>
-      <c r="AC1" t="str">
-        <v>RAS</v>
-      </c>
-      <c r="AD1" t="str">
-        <v>Others if any</v>
-      </c>
-      <c r="AE1" t="str">
-        <v>Total contribution by Garud in discounts</v>
-      </c>
-      <c r="AF1" t="str">
-        <v>Addtional Discount Given to Customer By Garud</v>
-      </c>
-      <c r="AG1" t="str">
-        <v>Total Garud Share of Discount passed on to customers</v>
-      </c>
-      <c r="AH1" t="str">
-        <v xml:space="preserve"> Scheme discount - Retail offtake</v>
-      </c>
-      <c r="AI1" t="str">
-        <v>Exchange</v>
-      </c>
-      <c r="AJ1" t="str">
-        <v>Corporate</v>
-      </c>
-      <c r="AK1" t="str">
-        <v>Intervention</v>
-      </c>
-      <c r="AL1" t="str">
-        <v>CSD</v>
-      </c>
-      <c r="AM1" t="str">
-        <v>Scrappage</v>
-      </c>
-      <c r="AN1" t="str">
-        <v>SSS</v>
-      </c>
-      <c r="AO1" t="str">
-        <v>Price Diffrance</v>
-      </c>
-      <c r="AP1" t="str">
-        <v>RAS</v>
-      </c>
-      <c r="AQ1" t="str">
-        <v>Other Scheme(any other additional support/speacial scheme if any)</v>
-      </c>
-      <c r="AR1" t="str">
-        <v>Total TML share of Discount passed on to the customers and to be claimed back from TML</v>
-      </c>
-      <c r="AS1" t="str">
-        <v xml:space="preserve"> Net Retained Margin After (Garud share of discount and  cash Disc)</v>
-      </c>
-      <c r="AT1" t="str">
-        <v>Percentage Margin Retained</v>
-      </c>
-      <c r="AU1" t="str">
-        <v xml:space="preserve"> Finance Income</v>
-      </c>
-      <c r="AV1" t="str">
-        <v>Insurance Income</v>
-      </c>
-      <c r="AW1" t="str">
-        <v>AMC Income</v>
-      </c>
-      <c r="AX1" t="str">
-        <v>Extended warranty Income</v>
-      </c>
-      <c r="AY1" t="str">
-        <v>Other Income  Registration &amp; Other Charges)</v>
-      </c>
-      <c r="AZ1" t="str">
-        <v>Accessories GP</v>
-      </c>
-      <c r="BA1" t="str">
-        <v>Total of Other Income</v>
-      </c>
-      <c r="BB1" t="str">
-        <v xml:space="preserve"> NRM (Retained DM+Other Income)</v>
-      </c>
-      <c r="BC1" t="str">
-        <v>Delivery Date</v>
-      </c>
-      <c r="BD1" t="str">
-        <v>Remarkes</v>
+        <v>Notes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:BD1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Capture and save all 20 form fields to Google Sheet
- saveCar() now sends all form fields: order no, dates, people, vehicle, pricing, discounts, income, remarks, stage
- Combine Garud scheme discount + additional discount when saving
- File upload handler sends all 20 columns to backend
- Excel template has all columns in Google Sheet order
- Data now flows completely from form → Google Sheet → other users
</commit_message>
<xml_diff>
--- a/public/nrm-template.xlsx
+++ b/public/nrm-template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:T1"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -419,81 +419,73 @@
     <col min="18" max="18" width="18.83203125" customWidth="1"/>
     <col min="19" max="19" width="18.83203125" customWidth="1"/>
     <col min="20" max="20" width="18.83203125" customWidth="1"/>
-    <col min="21" max="21" width="18.83203125" customWidth="1"/>
-    <col min="22" max="22" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Order No</v>
+        <v>Order Number</v>
       </c>
       <c r="B1" t="str">
-        <v>Booking Date</v>
+        <v>Invoice No</v>
       </c>
       <c r="C1" t="str">
-        <v>Customer</v>
+        <v>Invoice Date</v>
       </c>
       <c r="D1" t="str">
-        <v>Location</v>
+        <v>Customer Name</v>
       </c>
       <c r="E1" t="str">
-        <v>Executive</v>
+        <v>Chassis No</v>
       </c>
       <c r="F1" t="str">
         <v>Team Leader</v>
       </c>
       <c r="G1" t="str">
-        <v>Make</v>
+        <v>Location (Branch)</v>
       </c>
       <c r="H1" t="str">
+        <v>Executive Name</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Make (Product)</v>
+      </c>
+      <c r="J1" t="str">
         <v>Variant</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>Units</v>
       </c>
-      <c r="J1" t="str">
-        <v>Chassis No</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Allotment Date</v>
-      </c>
       <c r="L1" t="str">
-        <v>Invoice No</v>
+        <v>Pre GST Sales Price</v>
       </c>
       <c r="M1" t="str">
-        <v>Invoice Date</v>
+        <v>Pre GST Purchase Price</v>
       </c>
       <c r="N1" t="str">
+        <v>POD</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Garud Share of Discount</v>
+      </c>
+      <c r="P1" t="str">
+        <v>TML Share of Discount</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Other Income</v>
+      </c>
+      <c r="R1" t="str">
         <v>Delivery Date</v>
       </c>
-      <c r="O1" t="str">
-        <v>Sales Price</v>
-      </c>
-      <c r="P1" t="str">
-        <v>Purchase Price</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>POD</v>
-      </c>
-      <c r="R1" t="str">
-        <v>Scheme Discount</v>
-      </c>
       <c r="S1" t="str">
-        <v>Additional Discount</v>
+        <v>Remarks</v>
       </c>
       <c r="T1" t="str">
-        <v>TML Discount</v>
-      </c>
-      <c r="U1" t="str">
-        <v>Other Income</v>
-      </c>
-      <c r="V1" t="str">
-        <v>Notes</v>
+        <v>Stage (booked / allotted / sold / cancelled)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>